<commit_message>
Refine corporate bags dashboard per logistics feedback
Sort monthly trend chronologically, remove Tallas tab, rename Decisions
section to compra sugerida, and add Barquisimeto plus Web velocity rules.
Corporate plans now draw only from taller and transit with Maxi Tote capped
at 700 while store floor stock stays for retail presence.

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/PLANES_PEDIDO_CORPORATIVO_BOLSOS.xlsx
+++ b/PLANES_PEDIDO_CORPORATIVO_BOLSOS.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="46">
   <si>
     <t>Plan</t>
   </si>
@@ -48,16 +48,19 @@
     <t>Cant. pedido corporativo</t>
   </si>
   <si>
-    <t>Stock actual (tiendas+taller)</t>
-  </si>
-  <si>
-    <t>Arribo compra estimado</t>
-  </si>
-  <si>
-    <t>Stock disponible pre-pedido</t>
-  </si>
-  <si>
-    <t>Stock remanente post-pedido</t>
+    <t>Stock tiendas (no se toca)</t>
+  </si>
+  <si>
+    <t>Stock taller</t>
+  </si>
+  <si>
+    <t>Arribo compra (tránsito)</t>
+  </si>
+  <si>
+    <t>Pool corporativo (taller+tránsito)</t>
+  </si>
+  <si>
+    <t>Inventario total post-pedido</t>
   </si>
   <si>
     <t>Rotación mensual ajustada (und/mes)</t>
@@ -99,6 +102,18 @@
     <t>Proyección tienda VELA</t>
   </si>
   <si>
+    <t>Tienda nueva Barquisimeto</t>
+  </si>
+  <si>
+    <t>Canal Web repotenciado</t>
+  </si>
+  <si>
+    <t>Pedido corporativo</t>
+  </si>
+  <si>
+    <t>Tope Maxi Tote pedido</t>
+  </si>
+  <si>
     <t>Meses base rotación</t>
   </si>
   <si>
@@ -111,6 +126,15 @@
     <t>1.5× velocidad GRIE</t>
   </si>
   <si>
+    <t>Promedio mensual GRIE + Chacao + Tolón</t>
+  </si>
+  <si>
+    <t>Equivalente a 1 Chacao adicional</t>
+  </si>
+  <si>
+    <t>Solo taller + tránsito (stock tienda intacto)</t>
+  </si>
+  <si>
     <t>2026-03, 2026-04, 2026-05, 2026-06, 2026-07, 2026-08</t>
   </si>
   <si>
@@ -121,9 +145,6 @@
   </si>
   <si>
     <t>Stock tiendas</t>
-  </si>
-  <si>
-    <t>Stock taller</t>
   </si>
   <si>
     <t>Arribo compra</t>
@@ -492,10 +513,10 @@
         <v>2800</v>
       </c>
       <c r="C2">
-        <v>76.90000000000001</v>
+        <v>69</v>
       </c>
       <c r="D2">
-        <v>287.3</v>
+        <v>254</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -506,10 +527,10 @@
         <v>2800</v>
       </c>
       <c r="C3">
-        <v>9.199999999999999</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="D3">
-        <v>184.8</v>
+        <v>208.9</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -520,10 +541,10 @@
         <v>2800</v>
       </c>
       <c r="C4">
-        <v>109</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="D4">
-        <v>225.6</v>
+        <v>208.9</v>
       </c>
     </row>
   </sheetData>
@@ -533,10 +554,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -576,13 +597,16 @@
       <c r="M1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" spans="1:13">
+      <c r="N1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C2">
         <v>1500</v>
@@ -591,230 +615,245 @@
         <v>49</v>
       </c>
       <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
         <v>2350</v>
       </c>
-      <c r="F2">
-        <v>2399</v>
-      </c>
       <c r="G2">
+        <v>2350</v>
+      </c>
+      <c r="H2">
         <v>899</v>
       </c>
-      <c r="H2">
-        <v>350.8</v>
-      </c>
       <c r="I2">
-        <v>76.90000000000001</v>
+        <v>390.8</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="K2">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="L2">
-        <v>1451</v>
+        <v>0</v>
       </c>
       <c r="M2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
+        <v>1500</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C3">
         <v>600</v>
       </c>
       <c r="D3">
-        <v>761</v>
+        <v>134</v>
       </c>
       <c r="E3">
+        <v>627</v>
+      </c>
+      <c r="F3">
         <v>1000</v>
       </c>
-      <c r="F3">
-        <v>1761</v>
-      </c>
       <c r="G3">
+        <v>1627</v>
+      </c>
+      <c r="H3">
         <v>1161</v>
       </c>
-      <c r="H3">
-        <v>56.9</v>
-      </c>
       <c r="I3">
-        <v>612.1</v>
+        <v>64.7</v>
       </c>
       <c r="J3">
+        <v>538.3</v>
+      </c>
+      <c r="K3">
         <v>600</v>
       </c>
-      <c r="K3">
-        <v>0</v>
-      </c>
       <c r="L3">
         <v>0</v>
       </c>
       <c r="M3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:13">
+      <c r="N3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C4">
         <v>700</v>
       </c>
       <c r="D4">
-        <v>832</v>
+        <v>97</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>735</v>
       </c>
       <c r="F4">
-        <v>832</v>
+        <v>0</v>
       </c>
       <c r="G4">
+        <v>735</v>
+      </c>
+      <c r="H4">
         <v>132</v>
       </c>
-      <c r="H4">
-        <v>22.9</v>
-      </c>
       <c r="I4">
-        <v>172.9</v>
+        <v>25.6</v>
       </c>
       <c r="J4">
+        <v>154.7</v>
+      </c>
+      <c r="K4">
         <v>700</v>
       </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
       <c r="L4">
         <v>0</v>
       </c>
       <c r="M4">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:13">
+      <c r="N4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
       <c r="A5" t="s">
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C5">
-        <v>1025</v>
+        <v>1150</v>
       </c>
       <c r="D5">
         <v>49</v>
       </c>
       <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
         <v>2350</v>
       </c>
-      <c r="F5">
-        <v>2399</v>
-      </c>
       <c r="G5">
-        <v>1374</v>
+        <v>2350</v>
       </c>
       <c r="H5">
-        <v>350.8</v>
+        <v>1249</v>
       </c>
       <c r="I5">
-        <v>117.5</v>
+        <v>390.8</v>
       </c>
       <c r="J5">
-        <v>0</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="K5">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="L5">
-        <v>976</v>
+        <v>0</v>
       </c>
       <c r="M5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
+        <v>1150</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
       <c r="A6" t="s">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C6">
         <v>950</v>
       </c>
       <c r="D6">
-        <v>761</v>
+        <v>134</v>
       </c>
       <c r="E6">
+        <v>627</v>
+      </c>
+      <c r="F6">
         <v>1000</v>
       </c>
-      <c r="F6">
-        <v>1761</v>
-      </c>
       <c r="G6">
+        <v>1627</v>
+      </c>
+      <c r="H6">
         <v>811</v>
       </c>
-      <c r="H6">
-        <v>56.9</v>
-      </c>
       <c r="I6">
-        <v>427.6</v>
+        <v>64.7</v>
       </c>
       <c r="J6">
+        <v>376</v>
+      </c>
+      <c r="K6">
         <v>627</v>
       </c>
-      <c r="K6">
-        <v>134</v>
-      </c>
       <c r="L6">
-        <v>189</v>
+        <v>0</v>
       </c>
       <c r="M6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
+        <v>323</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
       <c r="A7" t="s">
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C7">
-        <v>825</v>
+        <v>700</v>
       </c>
       <c r="D7">
-        <v>832</v>
+        <v>97</v>
       </c>
       <c r="E7">
-        <v>0</v>
+        <v>735</v>
       </c>
       <c r="F7">
-        <v>832</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>7</v>
+        <v>735</v>
       </c>
       <c r="H7">
-        <v>22.9</v>
+        <v>132</v>
       </c>
       <c r="I7">
-        <v>9.199999999999999</v>
+        <v>25.6</v>
       </c>
       <c r="J7">
-        <v>735</v>
+        <v>154.7</v>
       </c>
       <c r="K7">
-        <v>90</v>
+        <v>700</v>
       </c>
       <c r="L7">
         <v>0</v>
@@ -822,127 +861,139 @@
       <c r="M7">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:13">
+      <c r="N7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
       <c r="A8" t="s">
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C8">
-        <v>1125</v>
+        <v>1150</v>
       </c>
       <c r="D8">
         <v>49</v>
       </c>
       <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
         <v>2350</v>
       </c>
-      <c r="F8">
-        <v>2399</v>
-      </c>
       <c r="G8">
-        <v>1274</v>
+        <v>2350</v>
       </c>
       <c r="H8">
-        <v>350.8</v>
+        <v>1249</v>
       </c>
       <c r="I8">
-        <v>109</v>
+        <v>390.8</v>
       </c>
       <c r="J8">
-        <v>0</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="K8">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="L8">
-        <v>1076</v>
+        <v>0</v>
       </c>
       <c r="M8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
+        <v>1150</v>
+      </c>
+      <c r="N8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
       <c r="A9" t="s">
         <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C9">
         <v>950</v>
       </c>
       <c r="D9">
-        <v>761</v>
+        <v>134</v>
       </c>
       <c r="E9">
+        <v>627</v>
+      </c>
+      <c r="F9">
         <v>1000</v>
       </c>
-      <c r="F9">
-        <v>1761</v>
-      </c>
       <c r="G9">
+        <v>1627</v>
+      </c>
+      <c r="H9">
         <v>811</v>
       </c>
-      <c r="H9">
-        <v>56.9</v>
-      </c>
       <c r="I9">
-        <v>427.6</v>
+        <v>64.7</v>
       </c>
       <c r="J9">
+        <v>376</v>
+      </c>
+      <c r="K9">
         <v>627</v>
       </c>
-      <c r="K9">
-        <v>134</v>
-      </c>
       <c r="L9">
-        <v>189</v>
+        <v>0</v>
       </c>
       <c r="M9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
+        <v>323</v>
+      </c>
+      <c r="N9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
       <c r="A10" t="s">
         <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C10">
-        <v>725</v>
+        <v>700</v>
       </c>
       <c r="D10">
-        <v>832</v>
+        <v>97</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>735</v>
       </c>
       <c r="F10">
-        <v>832</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>107</v>
+        <v>735</v>
       </c>
       <c r="H10">
-        <v>22.9</v>
+        <v>132</v>
       </c>
       <c r="I10">
-        <v>140.2</v>
+        <v>25.6</v>
       </c>
       <c r="J10">
-        <v>725</v>
+        <v>154.7</v>
       </c>
       <c r="K10">
-        <v>0</v>
+        <v>700</v>
       </c>
       <c r="L10">
         <v>0</v>
       </c>
       <c r="M10">
+        <v>0</v>
+      </c>
+      <c r="N10">
         <v>0</v>
       </c>
     </row>
@@ -953,20 +1004,20 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B2">
         <v>1.25</v>
@@ -974,34 +1025,66 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5">
-        <v>2800</v>
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
         <v>31</v>
+      </c>
+      <c r="B8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9">
+        <v>2800</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -1016,15 +1099,15 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="B1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="B2">
         <v>49</v>
@@ -1032,7 +1115,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -1040,7 +1123,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="B4">
         <v>2350</v>
@@ -1048,7 +1131,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="B5">
         <v>224.8</v>
@@ -1056,7 +1139,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="B6">
         <v>55.8</v>
@@ -1064,10 +1147,10 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="B7">
-        <v>350.8</v>
+        <v>390.8</v>
       </c>
     </row>
   </sheetData>
@@ -1082,15 +1165,15 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="B1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="B2">
         <v>134</v>
@@ -1098,7 +1181,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="B3">
         <v>627</v>
@@ -1106,7 +1189,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="B4">
         <v>1000</v>
@@ -1114,7 +1197,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="B5">
         <v>31.3</v>
@@ -1122,7 +1205,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="B6">
         <v>14.2</v>
@@ -1130,10 +1213,10 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="B7">
-        <v>56.9</v>
+        <v>64.7</v>
       </c>
     </row>
   </sheetData>
@@ -1148,15 +1231,15 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="B1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="B2">
         <v>97</v>
@@ -1164,7 +1247,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="B3">
         <v>735</v>
@@ -1172,7 +1255,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -1180,7 +1263,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="B5">
         <v>15.8</v>
@@ -1188,7 +1271,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="B6">
         <v>2.5</v>
@@ -1196,10 +1279,10 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="B7">
-        <v>22.9</v>
+        <v>25.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>